<commit_message>
Sanitize repo for public release
</commit_message>
<xml_diff>
--- a/docs/demo/client_brief_may2026.xlsx
+++ b/docs/demo/client_brief_may2026.xlsx
@@ -445,7 +445,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>act_366643171197739</t>
+          <t>act_000000000</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>102066921653934</t>
+          <t>000000000000000</t>
         </is>
       </c>
     </row>

</xml_diff>